<commit_message>
Store: 调整 Person 结构
</commit_message>
<xml_diff>
--- a/600.store/model.orm.xlsx
+++ b/600.store/model.orm.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12555" activeTab="4"/>
+    <workbookView windowWidth="28800" windowHeight="12555" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="配置" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="154">
   <si>
     <t>#变量名</t>
   </si>
@@ -357,15 +357,6 @@
   </si>
   <si>
     <t>身份证号</t>
-  </si>
-  <si>
-    <t>myself</t>
-  </si>
-  <si>
-    <t>「我」？</t>
-  </si>
-  <si>
-    <t>是否为资产库所有者。有且仅有一个</t>
   </si>
   <si>
     <t>deleted</t>
@@ -2672,7 +2663,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="3" width="9" style="1"/>
@@ -3036,9 +3027,9 @@
       <c r="N13" s="33"/>
       <c r="O13" s="9"/>
     </row>
-    <row r="14" s="1" customFormat="1" ht="40.5" spans="1:15">
+    <row r="14" s="1" customFormat="1" ht="15" spans="1:15">
       <c r="A14" s="9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -3049,11 +3040,13 @@
       <c r="F14" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="G14" s="5"/>
+      <c r="G14" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="H14" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="I14" s="31" t="s">
+      <c r="I14" s="35" t="s">
         <v>46</v>
       </c>
       <c r="J14" s="32"/>
@@ -3066,34 +3059,20 @@
       <c r="O14" s="9"/>
     </row>
     <row r="15" s="1" customFormat="1" ht="15" spans="1:15">
-      <c r="A15" s="9">
-        <v>8</v>
-      </c>
+      <c r="A15" s="9"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
-      <c r="D15" s="5" t="s">
-        <v>116</v>
-      </c>
+      <c r="D15" s="5"/>
       <c r="E15" s="9"/>
-      <c r="F15" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="I15" s="35" t="s">
-        <v>46</v>
-      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="35"/>
       <c r="J15" s="32"/>
       <c r="K15" s="9"/>
       <c r="L15" s="33"/>
       <c r="M15" s="5"/>
-      <c r="N15" s="33" t="s">
-        <v>118</v>
-      </c>
+      <c r="N15" s="33"/>
       <c r="O15" s="9"/>
     </row>
     <row r="16" s="1" customFormat="1" ht="15" spans="1:15">
@@ -3147,106 +3126,106 @@
       <c r="N18" s="33"/>
       <c r="O18" s="9"/>
     </row>
-    <row r="19" s="1" customFormat="1" ht="15" spans="1:15">
+    <row r="19" s="1" customFormat="1" spans="1:15">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
-      <c r="D19" s="5"/>
+      <c r="D19" s="9"/>
       <c r="E19" s="9"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
       <c r="H19" s="9"/>
-      <c r="I19" s="35"/>
-      <c r="J19" s="32"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
       <c r="K19" s="9"/>
       <c r="L19" s="33"/>
       <c r="M19" s="5"/>
       <c r="N19" s="33"/>
       <c r="O19" s="9"/>
     </row>
-    <row r="20" s="1" customFormat="1" spans="1:15">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-      <c r="L20" s="33"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="33"/>
-      <c r="O20" s="9"/>
+    <row r="20" s="3" customFormat="1" spans="1:15">
+      <c r="A20" s="11"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="46"/>
     </row>
     <row r="21" s="3" customFormat="1" spans="1:15">
-      <c r="A21" s="11"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12"/>
-      <c r="I21" s="12"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
-      <c r="L21" s="12"/>
-      <c r="M21" s="12"/>
-      <c r="N21" s="12"/>
-      <c r="O21" s="46"/>
+      <c r="A21" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="14"/>
+      <c r="L21" s="14"/>
+      <c r="M21" s="14"/>
+      <c r="N21" s="14"/>
+      <c r="O21" s="47"/>
     </row>
     <row r="22" s="3" customFormat="1" spans="1:15">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="C22" s="17"/>
+      <c r="D22" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
-      <c r="M22" s="14"/>
-      <c r="N22" s="14"/>
-      <c r="O22" s="47"/>
+      <c r="K22" s="36"/>
+      <c r="L22" s="36"/>
+      <c r="M22" s="36"/>
+      <c r="N22" s="36"/>
+      <c r="O22" s="17"/>
     </row>
     <row r="23" s="3" customFormat="1" spans="1:15">
-      <c r="A23" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B23" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="F23" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="G23" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="H23" s="15"/>
-      <c r="I23" s="15"/>
-      <c r="J23" s="16" t="s">
-        <v>122</v>
-      </c>
-      <c r="K23" s="36"/>
-      <c r="L23" s="36"/>
-      <c r="M23" s="36"/>
-      <c r="N23" s="36"/>
-      <c r="O23" s="17"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="38"/>
+      <c r="K23" s="39"/>
+      <c r="L23" s="39"/>
+      <c r="M23" s="39"/>
+      <c r="N23" s="39"/>
+      <c r="O23" s="48"/>
     </row>
     <row r="24" s="3" customFormat="1" spans="1:15">
       <c r="A24" s="18"/>
@@ -3299,75 +3278,81 @@
       <c r="N26" s="39"/>
       <c r="O26" s="48"/>
     </row>
-    <row r="27" s="3" customFormat="1" spans="1:15">
-      <c r="A27" s="18"/>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="39"/>
-      <c r="I27" s="48"/>
-      <c r="J27" s="38"/>
-      <c r="K27" s="39"/>
-      <c r="L27" s="39"/>
-      <c r="M27" s="39"/>
-      <c r="N27" s="39"/>
-      <c r="O27" s="48"/>
+    <row r="27" s="1" customFormat="1" spans="1:15">
+      <c r="A27" s="20"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="21"/>
+      <c r="L27" s="21"/>
+      <c r="M27" s="21"/>
+      <c r="N27" s="21"/>
+      <c r="O27" s="49"/>
     </row>
     <row r="28" s="1" customFormat="1" spans="1:15">
-      <c r="A28" s="20"/>
-      <c r="B28" s="21"/>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="21"/>
-      <c r="J28" s="21"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="21"/>
-      <c r="M28" s="21"/>
-      <c r="N28" s="21"/>
-      <c r="O28" s="49"/>
+      <c r="A28" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="8"/>
     </row>
     <row r="29" s="1" customFormat="1" spans="1:15">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="22"/>
+      <c r="B29" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C29" s="4"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="8"/>
-      <c r="K29" s="8"/>
-      <c r="L29" s="8"/>
-      <c r="M29" s="8"/>
-      <c r="N29" s="8"/>
-      <c r="O29" s="8"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
     </row>
     <row r="30" s="1" customFormat="1" spans="1:15">
       <c r="A30" s="22"/>
       <c r="B30" s="4" t="s">
-        <v>124</v>
+        <v>54</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
       <c r="F30" s="4" t="s">
-        <v>125</v>
+        <v>56</v>
       </c>
       <c r="G30" s="5"/>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
       <c r="J30" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K30" s="4"/>
       <c r="L30" s="5"/>
@@ -3378,20 +3363,18 @@
     <row r="31" s="1" customFormat="1" spans="1:15">
       <c r="A31" s="22"/>
       <c r="B31" s="4" t="s">
-        <v>54</v>
+        <v>125</v>
       </c>
       <c r="C31" s="4"/>
       <c r="D31" s="5"/>
       <c r="E31" s="5"/>
       <c r="F31" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="4" t="s">
-        <v>127</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
+      <c r="J31" s="4"/>
       <c r="K31" s="4"/>
       <c r="L31" s="5"/>
       <c r="M31" s="5"/>
@@ -3401,18 +3384,18 @@
     <row r="32" s="1" customFormat="1" spans="1:15">
       <c r="A32" s="22"/>
       <c r="B32" s="4" t="s">
-        <v>128</v>
+        <v>87</v>
       </c>
       <c r="C32" s="4"/>
       <c r="D32" s="5"/>
       <c r="E32" s="5"/>
-      <c r="F32" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="G32" s="9"/>
-      <c r="H32" s="9"/>
-      <c r="I32" s="9"/>
-      <c r="J32" s="4"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="4" t="s">
+        <v>86</v>
+      </c>
       <c r="K32" s="4"/>
       <c r="L32" s="5"/>
       <c r="M32" s="5"/>
@@ -3421,92 +3404,88 @@
     </row>
     <row r="33" s="1" customFormat="1" spans="1:15">
       <c r="A33" s="22"/>
-      <c r="B33" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C33" s="4"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K33" s="4"/>
-      <c r="L33" s="5"/>
-      <c r="M33" s="5"/>
-      <c r="N33" s="5"/>
-      <c r="O33" s="5"/>
+      <c r="B33" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="23"/>
+      <c r="J33" s="40"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="40"/>
+      <c r="M33" s="50"/>
+      <c r="N33" s="50"/>
+      <c r="O33" s="41"/>
     </row>
     <row r="34" s="1" customFormat="1" spans="1:15">
       <c r="A34" s="22"/>
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F34" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C34" s="23"/>
-      <c r="D34" s="23"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="23"/>
-      <c r="I34" s="23"/>
-      <c r="J34" s="40"/>
-      <c r="K34" s="41"/>
-      <c r="L34" s="40"/>
-      <c r="M34" s="50"/>
-      <c r="N34" s="50"/>
-      <c r="O34" s="41"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
     </row>
     <row r="35" s="1" customFormat="1" spans="1:15">
       <c r="A35" s="22"/>
-      <c r="B35" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="4"/>
-      <c r="M35" s="4"/>
-      <c r="N35" s="4"/>
-      <c r="O35" s="4"/>
+      <c r="B35" s="9">
+        <v>1</v>
+      </c>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
     </row>
     <row r="36" s="1" customFormat="1" spans="1:15">
-      <c r="A36" s="22"/>
-      <c r="B36" s="9">
-        <v>1</v>
-      </c>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
+      <c r="A36" s="24"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="25"/>
       <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="9"/>
-      <c r="K36" s="9"/>
-      <c r="L36" s="9"/>
-      <c r="M36" s="9"/>
-      <c r="N36" s="9"/>
-      <c r="O36" s="9"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="30"/>
+      <c r="J36" s="42"/>
+      <c r="K36" s="43"/>
+      <c r="L36" s="42"/>
+      <c r="M36" s="51"/>
+      <c r="N36" s="51"/>
+      <c r="O36" s="43"/>
     </row>
     <row r="37" s="1" customFormat="1" spans="1:15">
-      <c r="A37" s="24"/>
+      <c r="A37" s="26"/>
       <c r="B37" s="9"/>
       <c r="C37" s="6"/>
       <c r="D37" s="25"/>
@@ -3523,38 +3502,44 @@
       <c r="O37" s="43"/>
     </row>
     <row r="38" s="1" customFormat="1" spans="1:15">
-      <c r="A38" s="26"/>
-      <c r="B38" s="9"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="25"/>
+      <c r="A38" s="22"/>
+      <c r="B38" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C38" s="4"/>
+      <c r="D38" s="5"/>
       <c r="E38" s="5"/>
-      <c r="F38" s="6"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="6"/>
-      <c r="I38" s="30"/>
-      <c r="J38" s="42"/>
-      <c r="K38" s="43"/>
-      <c r="L38" s="42"/>
-      <c r="M38" s="51"/>
-      <c r="N38" s="51"/>
-      <c r="O38" s="43"/>
+      <c r="F38" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="K38" s="4"/>
+      <c r="L38" s="5"/>
+      <c r="M38" s="5"/>
+      <c r="N38" s="5"/>
+      <c r="O38" s="5"/>
     </row>
     <row r="39" s="1" customFormat="1" spans="1:15">
       <c r="A39" s="22"/>
       <c r="B39" s="4" t="s">
-        <v>124</v>
+        <v>54</v>
       </c>
       <c r="C39" s="4"/>
       <c r="D39" s="5"/>
       <c r="E39" s="5"/>
       <c r="F39" s="4" t="s">
-        <v>125</v>
+        <v>56</v>
       </c>
       <c r="G39" s="5"/>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
       <c r="J39" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K39" s="4"/>
       <c r="L39" s="5"/>
@@ -3565,20 +3550,18 @@
     <row r="40" s="1" customFormat="1" spans="1:15">
       <c r="A40" s="22"/>
       <c r="B40" s="4" t="s">
-        <v>54</v>
+        <v>125</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
       <c r="F40" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="4" t="s">
-        <v>127</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
+      <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="5"/>
       <c r="M40" s="5"/>
@@ -3588,18 +3571,18 @@
     <row r="41" s="1" customFormat="1" spans="1:15">
       <c r="A41" s="22"/>
       <c r="B41" s="4" t="s">
-        <v>128</v>
+        <v>87</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
-      <c r="F41" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="G41" s="9"/>
-      <c r="H41" s="9"/>
-      <c r="I41" s="9"/>
-      <c r="J41" s="4"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="4" t="s">
+        <v>86</v>
+      </c>
       <c r="K41" s="4"/>
       <c r="L41" s="5"/>
       <c r="M41" s="5"/>
@@ -3608,92 +3591,88 @@
     </row>
     <row r="42" s="1" customFormat="1" spans="1:15">
       <c r="A42" s="22"/>
-      <c r="B42" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C42" s="4"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5"/>
-      <c r="J42" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K42" s="4"/>
-      <c r="L42" s="5"/>
-      <c r="M42" s="5"/>
-      <c r="N42" s="5"/>
-      <c r="O42" s="5"/>
+      <c r="B42" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="C42" s="23"/>
+      <c r="D42" s="23"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="23"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="40"/>
+      <c r="K42" s="41"/>
+      <c r="L42" s="40"/>
+      <c r="M42" s="50"/>
+      <c r="N42" s="50"/>
+      <c r="O42" s="41"/>
     </row>
     <row r="43" s="1" customFormat="1" spans="1:15">
       <c r="A43" s="22"/>
-      <c r="B43" s="23" t="s">
+      <c r="B43" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F43" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C43" s="23"/>
-      <c r="D43" s="23"/>
-      <c r="E43" s="23"/>
-      <c r="F43" s="23"/>
-      <c r="G43" s="23"/>
-      <c r="H43" s="23"/>
-      <c r="I43" s="23"/>
-      <c r="J43" s="40"/>
-      <c r="K43" s="41"/>
-      <c r="L43" s="40"/>
-      <c r="M43" s="50"/>
-      <c r="N43" s="50"/>
-      <c r="O43" s="41"/>
+      <c r="G43" s="4"/>
+      <c r="H43" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="4"/>
+      <c r="L43" s="4"/>
+      <c r="M43" s="4"/>
+      <c r="N43" s="4"/>
+      <c r="O43" s="4"/>
     </row>
     <row r="44" s="1" customFormat="1" spans="1:15">
       <c r="A44" s="22"/>
-      <c r="B44" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="I44" s="4"/>
-      <c r="J44" s="4"/>
-      <c r="K44" s="4"/>
-      <c r="L44" s="4"/>
-      <c r="M44" s="4"/>
-      <c r="N44" s="4"/>
-      <c r="O44" s="4"/>
+      <c r="B44" s="9">
+        <v>1</v>
+      </c>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="9"/>
+      <c r="K44" s="9"/>
+      <c r="L44" s="9"/>
+      <c r="M44" s="9"/>
+      <c r="N44" s="9"/>
+      <c r="O44" s="9"/>
     </row>
     <row r="45" s="1" customFormat="1" spans="1:15">
-      <c r="A45" s="22"/>
-      <c r="B45" s="9">
-        <v>1</v>
-      </c>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5"/>
+      <c r="A45" s="24"/>
+      <c r="B45" s="9"/>
+      <c r="C45" s="6"/>
+      <c r="D45" s="25"/>
       <c r="E45" s="5"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-      <c r="I45" s="5"/>
-      <c r="J45" s="9"/>
-      <c r="K45" s="9"/>
-      <c r="L45" s="9"/>
-      <c r="M45" s="9"/>
-      <c r="N45" s="9"/>
-      <c r="O45" s="9"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="30"/>
+      <c r="H45" s="6"/>
+      <c r="I45" s="30"/>
+      <c r="J45" s="42"/>
+      <c r="K45" s="43"/>
+      <c r="L45" s="42"/>
+      <c r="M45" s="51"/>
+      <c r="N45" s="51"/>
+      <c r="O45" s="43"/>
     </row>
     <row r="46" s="1" customFormat="1" spans="1:15">
-      <c r="A46" s="24"/>
+      <c r="A46" s="26"/>
       <c r="B46" s="9"/>
       <c r="C46" s="6"/>
       <c r="D46" s="25"/>
@@ -3708,23 +3687,6 @@
       <c r="M46" s="51"/>
       <c r="N46" s="51"/>
       <c r="O46" s="43"/>
-    </row>
-    <row r="47" s="1" customFormat="1" spans="1:15">
-      <c r="A47" s="26"/>
-      <c r="B47" s="9"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="25"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="6"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="6"/>
-      <c r="I47" s="30"/>
-      <c r="J47" s="42"/>
-      <c r="K47" s="43"/>
-      <c r="L47" s="42"/>
-      <c r="M47" s="51"/>
-      <c r="N47" s="51"/>
-      <c r="O47" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="118">
@@ -3741,8 +3703,11 @@
     <mergeCell ref="D4:O4"/>
     <mergeCell ref="A5:O5"/>
     <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A20:O20"/>
     <mergeCell ref="A21:O21"/>
-    <mergeCell ref="A22:O22"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="J22:O22"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="G23:I23"/>
     <mergeCell ref="J23:O23"/>
@@ -3755,11 +3720,13 @@
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="G26:I26"/>
     <mergeCell ref="J26:O26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="J27:O27"/>
+    <mergeCell ref="A27:O27"/>
     <mergeCell ref="A28:O28"/>
-    <mergeCell ref="A29:O29"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="L29:O29"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="G30:I30"/>
@@ -3771,15 +3738,15 @@
     <mergeCell ref="J31:K31"/>
     <mergeCell ref="L31:O31"/>
     <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="D32:I32"/>
     <mergeCell ref="J32:K32"/>
     <mergeCell ref="L32:O32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="B33:I33"/>
     <mergeCell ref="J33:K33"/>
     <mergeCell ref="L33:O33"/>
-    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H34:I34"/>
     <mergeCell ref="J34:K34"/>
     <mergeCell ref="L34:O34"/>
     <mergeCell ref="C35:D35"/>
@@ -3797,9 +3764,9 @@
     <mergeCell ref="H37:I37"/>
     <mergeCell ref="J37:K37"/>
     <mergeCell ref="L37:O37"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="G38:I38"/>
     <mergeCell ref="J38:K38"/>
     <mergeCell ref="L38:O38"/>
     <mergeCell ref="B39:C39"/>
@@ -3813,15 +3780,15 @@
     <mergeCell ref="J40:K40"/>
     <mergeCell ref="L40:O40"/>
     <mergeCell ref="B41:C41"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="G41:I41"/>
+    <mergeCell ref="D41:I41"/>
     <mergeCell ref="J41:K41"/>
     <mergeCell ref="L41:O41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="D42:I42"/>
+    <mergeCell ref="B42:I42"/>
     <mergeCell ref="J42:K42"/>
     <mergeCell ref="L42:O42"/>
-    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="H43:I43"/>
     <mergeCell ref="J43:K43"/>
     <mergeCell ref="L43:O43"/>
     <mergeCell ref="C44:D44"/>
@@ -3839,13 +3806,8 @@
     <mergeCell ref="H46:I46"/>
     <mergeCell ref="J46:K46"/>
     <mergeCell ref="L46:O46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="J47:K47"/>
-    <mergeCell ref="L47:O47"/>
-    <mergeCell ref="A30:A38"/>
-    <mergeCell ref="A39:A47"/>
+    <mergeCell ref="A29:A37"/>
+    <mergeCell ref="A38:A46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -3879,7 +3841,7 @@
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="5" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
@@ -3887,7 +3849,7 @@
         <v>82</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="I1" s="25"/>
       <c r="J1" s="25"/>
@@ -3904,7 +3866,7 @@
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -3948,7 +3910,7 @@
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
       <c r="D4" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E4" s="25"/>
       <c r="F4" s="25"/>
@@ -4085,11 +4047,11 @@
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="9" t="s">
@@ -4114,11 +4076,11 @@
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="G10" s="5"/>
       <c r="H10" s="9" t="s">
@@ -4143,11 +4105,11 @@
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
       <c r="D11" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G11" s="5"/>
       <c r="H11" s="9" t="s">
@@ -4341,7 +4303,7 @@
     </row>
     <row r="22" s="3" customFormat="1" spans="1:15">
       <c r="A22" s="13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
@@ -4363,7 +4325,7 @@
         <v>29</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C23" s="17"/>
       <c r="D23" s="16" t="s">
@@ -4376,12 +4338,12 @@
         <v>56</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="H23" s="15"/>
       <c r="I23" s="15"/>
       <c r="J23" s="16" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K23" s="36"/>
       <c r="L23" s="36"/>
@@ -4394,16 +4356,16 @@
         <v>1</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C24" s="19"/>
       <c r="D24" s="18" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E24" s="27"/>
       <c r="F24" s="27"/>
       <c r="G24" s="28" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="H24" s="29"/>
       <c r="I24" s="37"/>
@@ -4484,7 +4446,7 @@
     </row>
     <row r="29" s="1" customFormat="1" spans="1:15">
       <c r="A29" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -4506,23 +4468,23 @@
         <v>1</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="E30" s="5"/>
       <c r="F30" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
       <c r="J30" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="K30" s="4"/>
       <c r="L30" s="5" t="s">
@@ -4539,7 +4501,7 @@
       </c>
       <c r="C31" s="4"/>
       <c r="D31" s="5" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E31" s="5"/>
       <c r="F31" s="4" t="s">
@@ -4549,11 +4511,11 @@
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
       <c r="J31" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="K31" s="4"/>
       <c r="L31" s="5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
@@ -4562,13 +4524,13 @@
     <row r="32" s="1" customFormat="1" spans="1:15">
       <c r="A32" s="22"/>
       <c r="B32" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C32" s="4"/>
       <c r="D32" s="5"/>
       <c r="E32" s="5"/>
       <c r="F32" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
@@ -4597,7 +4559,7 @@
       </c>
       <c r="K33" s="4"/>
       <c r="L33" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="M33" s="5"/>
       <c r="N33" s="5"/>
@@ -4606,7 +4568,7 @@
     <row r="34" s="1" customFormat="1" spans="1:15">
       <c r="A34" s="22"/>
       <c r="B34" s="23" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C34" s="23"/>
       <c r="D34" s="23"/>
@@ -4628,18 +4590,18 @@
         <v>29</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D35" s="4"/>
       <c r="E35" s="4" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
@@ -4655,7 +4617,7 @@
         <v>1</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D36" s="5"/>
       <c r="E36" s="5"/>
@@ -4711,23 +4673,23 @@
         <v>2</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C39" s="4"/>
       <c r="D39" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E39" s="5"/>
       <c r="F39" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
       <c r="J39" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="K39" s="4"/>
       <c r="L39" s="5" t="s">
@@ -4744,7 +4706,7 @@
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E40" s="5"/>
       <c r="F40" s="4" t="s">
@@ -4754,11 +4716,11 @@
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
       <c r="J40" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="K40" s="4"/>
       <c r="L40" s="5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="M40" s="5"/>
       <c r="N40" s="5"/>
@@ -4767,13 +4729,13 @@
     <row r="41" s="1" customFormat="1" spans="1:15">
       <c r="A41" s="22"/>
       <c r="B41" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
       <c r="F41" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G41" s="9"/>
       <c r="H41" s="9"/>
@@ -4802,7 +4764,7 @@
       </c>
       <c r="K42" s="4"/>
       <c r="L42" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="M42" s="5"/>
       <c r="N42" s="5"/>
@@ -4811,7 +4773,7 @@
     <row r="43" s="1" customFormat="1" spans="1:15">
       <c r="A43" s="22"/>
       <c r="B43" s="23" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C43" s="23"/>
       <c r="D43" s="23"/>
@@ -4833,18 +4795,18 @@
         <v>29</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="4" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="G44" s="4"/>
       <c r="H44" s="4" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I44" s="4"/>
       <c r="J44" s="4"/>
@@ -4860,7 +4822,7 @@
         <v>1</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D45" s="5"/>
       <c r="E45" s="5"/>

</xml_diff>